<commit_message>
Rebuild order database from the five specified tabs using first cell entries
</commit_message>
<xml_diff>
--- a/downloads/AutoReport_query_template.xlsx
+++ b/downloads/AutoReport_query_template.xlsx
@@ -10,7 +10,7 @@
     <sheet name="待查詢資料" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'待查詢資料'!$A$1:$D$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'待查詢資料'!$A$1:$D$16</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -425,11 +425,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
   </cols>
@@ -467,61 +467,151 @@
       <c r="D2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr"/>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>98000320-107</t>
-        </is>
-      </c>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>C514-260400001</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr"/>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>FP-D01304BE11</t>
-        </is>
-      </c>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>C533-250800002</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr"/>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>找不到的料號</t>
-        </is>
-      </c>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>C533-251200001</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr"/>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>98000239-106</t>
-        </is>
-      </c>
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>C515-251100001</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>C515-250300004</t>
+          <t>C516-626070202</t>
         </is>
       </c>
       <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr"/>
-      <c r="D7" t="inlineStr">
+      <c r="D7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>626090006</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr"/>
+      <c r="C8" t="inlineStr"/>
+      <c r="D8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>C630-626080041</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr"/>
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr"/>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>98000320-107</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr"/>
+      <c r="D10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>C533-260100003</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr"/>
+      <c r="C11" t="inlineStr"/>
+      <c r="D11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>C630-626080043</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr"/>
+      <c r="C12" t="inlineStr"/>
+      <c r="D12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>C510-260500009</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr"/>
+      <c r="C13" t="inlineStr"/>
+      <c r="D13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr"/>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>找不到的料號</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr"/>
+      <c r="D14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>C515-250300004</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr"/>
+      <c r="C15" t="inlineStr"/>
+      <c r="D15" t="inlineStr">
         <is>
           <t>Synaptics</t>
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>C515-251100004</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr"/>
+      <c r="C16" t="inlineStr"/>
+      <c r="D16" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D7"/>
+  <autoFilter ref="A1:D16"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>